<commit_message>
Add GitLab CI config and update results file
</commit_message>
<xml_diff>
--- a/tippningar.xlsx
+++ b/tippningar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ellabacklund/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ellabacklund/Claude_project/vm-tippning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B5B567-4595-424A-AF83-D7CBE6C86FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F838CD4E-EAA5-EE4F-9544-DA017E687F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="600" windowWidth="28240" windowHeight="15880" xr2:uid="{16FA151C-8F69-3E42-B82E-CE219F9BC60A}"/>
+    <workbookView xWindow="280" yWindow="600" windowWidth="28240" windowHeight="15820" xr2:uid="{16FA151C-8F69-3E42-B82E-CE219F9BC60A}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="37">
   <si>
     <t>Vinst</t>
   </si>
@@ -126,6 +126,30 @@
   </si>
   <si>
     <t>Kanada</t>
+  </si>
+  <si>
+    <t>Nils</t>
+  </si>
+  <si>
+    <t>Erland</t>
+  </si>
+  <si>
+    <t>Algeriet</t>
+  </si>
+  <si>
+    <t>Pappa</t>
+  </si>
+  <si>
+    <t>Argenina</t>
+  </si>
+  <si>
+    <t>Axel</t>
+  </si>
+  <si>
+    <t>Karin</t>
+  </si>
+  <si>
+    <t>Sydkorea</t>
   </si>
 </sst>
 </file>
@@ -512,10 +536,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FBA6A90-EBA8-D348-A40C-CFBB2BF06EF7}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
@@ -531,8 +555,23 @@
       <c r="J1" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -551,8 +590,21 @@
       <c r="J2" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="L2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="T2" s="1"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -571,8 +623,20 @@
       <c r="J4" t="s">
         <v>2</v>
       </c>
+      <c r="L4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" t="s">
+        <v>2</v>
+      </c>
+      <c r="P4" t="s">
+        <v>7</v>
+      </c>
+      <c r="R4" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -591,8 +655,20 @@
       <c r="J6" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="L6" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
@@ -608,8 +684,20 @@
       <c r="J7" t="s">
         <v>22</v>
       </c>
+      <c r="L7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" t="s">
+        <v>8</v>
+      </c>
+      <c r="P7" t="s">
+        <v>10</v>
+      </c>
+      <c r="R7" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -628,8 +716,20 @@
       <c r="J9" t="s">
         <v>11</v>
       </c>
+      <c r="L9" t="s">
+        <v>7</v>
+      </c>
+      <c r="N9" t="s">
+        <v>14</v>
+      </c>
+      <c r="P9" t="s">
+        <v>2</v>
+      </c>
+      <c r="R9" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>11</v>
       </c>
@@ -645,8 +745,20 @@
       <c r="J10" t="s">
         <v>7</v>
       </c>
+      <c r="L10" t="s">
+        <v>20</v>
+      </c>
+      <c r="N10" t="s">
+        <v>7</v>
+      </c>
+      <c r="P10" t="s">
+        <v>11</v>
+      </c>
+      <c r="R10" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>12</v>
       </c>
@@ -657,13 +769,25 @@
         <v>20</v>
       </c>
       <c r="H11" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="J11" t="s">
         <v>27</v>
       </c>
+      <c r="L11" t="s">
+        <v>14</v>
+      </c>
+      <c r="N11" t="s">
+        <v>11</v>
+      </c>
+      <c r="P11" t="s">
+        <v>8</v>
+      </c>
+      <c r="R11" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>13</v>
       </c>
@@ -678,9 +802,22 @@
       </c>
       <c r="J12" t="s">
         <v>28</v>
+      </c>
+      <c r="L12" t="s">
+        <v>11</v>
+      </c>
+      <c r="N12" t="s">
+        <v>31</v>
+      </c>
+      <c r="P12" t="s">
+        <v>15</v>
+      </c>
+      <c r="R12" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bytt plats på farfars trea
</commit_message>
<xml_diff>
--- a/tippningar.xlsx
+++ b/tippningar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ellabacklund/Claude_project/vm-tippning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAFC884-890E-0249-89C0-DA970F7E5CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C5EC0A-648B-CA41-B19C-5E7F0EB5E1CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="600" windowWidth="28240" windowHeight="15820" xr2:uid="{16FA151C-8F69-3E42-B82E-CE219F9BC60A}"/>
   </bookViews>
@@ -642,9 +642,10 @@
       <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
         <v>14</v>
       </c>
@@ -674,8 +675,8 @@
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B7" s="1" t="s">
-        <v>7</v>
+      <c r="B7" t="s">
+        <v>10</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>

</xml_diff>